<commit_message>
Split stok: hidup vs frozen/mati terpisah. 6 kategori stok (+ campuran diskon)
</commit_message>
<xml_diff>
--- a/Template Catatan Bulanan - VhannyLobster.xlsx
+++ b/Template Catatan Bulanan - VhannyLobster.xlsx
@@ -71,7 +71,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -93,11 +93,17 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -118,6 +124,14 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -663,7 +677,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -795,7 +808,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -898,7 +910,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -960,152 +971,202 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Salatiga</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Salatiga (hidup)</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n">
         <v>130</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2">
+      <c r="C2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="10">
         <f>B2+C2-D2-E2</f>
         <v/>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Lobster hidup</t>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>Lobster hidup, sisa batch 300kg</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Boyolali</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Boyolali (hidup)</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
         <v>145</v>
       </c>
-      <c r="C3" s="7" t="n">
-        <v>250</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6">
+      <c r="C3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="10">
         <f>B3+C3-D3-E3</f>
         <v/>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>145 hidup + 250 frozen</t>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Lobster hidup, sisa batch 400kg</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Jogja</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="C4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Boyolali (frozen baru)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="10">
         <f>B4+C4-D4-E4</f>
         <v/>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Lobster hidup</t>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Pembelian 26 Jul, 250kg frozen</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Bekasi</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="6">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Jogja (hidup)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="10">
         <f>B5+C5-D5-E5</f>
         <v/>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Fresh/frozen</t>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Lobster hidup, sisa batch 19kg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Bekasi (fresh/frozen)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11">
+        <f>B6+C6-D6-E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Sisa dari 30kg. 2kg frozen terjual 27 Jul</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Campuran (mati/frozen)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="10">
+        <f>B7+C7-D7-E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Harga jual diskon Rp 180rb/kg. 6kg terjual 26 Jul. Sisa 25kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="9">
-        <f>SUM(B2:B5)</f>
+      <c r="B8" s="13">
+        <f>SUM(B2:B7)</f>
         <v/>
       </c>
-      <c r="C6" s="9">
-        <f>SUM(C2:C5)</f>
+      <c r="C8" s="13">
+        <f>SUM(C2:C7)</f>
         <v/>
       </c>
-      <c r="D6" s="9">
-        <f>SUM(D2:D5)</f>
+      <c r="D8" s="13">
+        <f>SUM(D2:D7)</f>
         <v/>
       </c>
-      <c r="E6" s="9">
-        <f>SUM(E2:E5)</f>
+      <c r="E8" s="13">
+        <f>SUM(E2:E7)</f>
         <v/>
       </c>
-      <c r="F6" s="9">
-        <f>SUM(F2:F5)</f>
+      <c r="F8" s="13">
+        <f>SUM(F2:F7)</f>
         <v/>
       </c>
-      <c r="G6" s="9">
-        <f>SUM(G2:G5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>PETUNJUK:</t>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Stok akhir otomatis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Entry TRX-048 (6kg mati Rp1.080.000) + TRX-049 (2kg frozen Rp360.000) + deduct 31kg from Boyolali
</commit_message>
<xml_diff>
--- a/Template Catatan Bulanan - VhannyLobster.xlsx
+++ b/Template Catatan Bulanan - VhannyLobster.xlsx
@@ -994,7 +994,7 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>Lobster hidup, sisa batch 300kg</t>
+          <t>Lobster hidup</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F3" s="10">
         <f>B3+C3-D3-E3</f>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>Lobster hidup, sisa batch 400kg</t>
+          <t>31kg mati → pindah ke campuran. Sisa 114kg hidup</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>Pembelian 26 Jul, 250kg frozen</t>
+          <t>Pembelian 26 Jul</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Lobster hidup, sisa batch 19kg</t>
+          <t>Lobster hidup</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Sisa dari 30kg. 2kg frozen terjual 27 Jul</t>
+          <t>2kg frozen terjual 27 Jul</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Harga jual diskon Rp 180rb/kg. 6kg terjual 26 Jul. Sisa 25kg</t>
+          <t>Dari Boyolali. 6kg terjual 26 Jul. Sisa 25kg @Rp180rb</t>
         </is>
       </c>
     </row>
@@ -1164,11 +1164,7 @@
         <f>SUM(F2:F7)</f>
         <v/>
       </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Stok akhir otomatis</t>
-        </is>
-      </c>
+      <c r="G8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">

</xml_diff>